<commit_message>
Done with day 25 and 26
</commit_message>
<xml_diff>
--- a/3.Problems for Revision.xlsx
+++ b/3.Problems for Revision.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="67">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -212,6 +212,18 @@
   </si>
   <si>
     <t xml:space="preserve">Practice Sorting 2D Array acc to first or last element</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My Clalender II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/my-calendar-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25 &amp; 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line Sweep Algo explained</t>
   </si>
 </sst>
 </file>
@@ -221,7 +233,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,12 +330,6 @@
       <family val="4"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Comic Sans MS"/>
-      <family val="4"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -428,6 +434,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -442,10 +452,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1159,7 +1165,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="18.03"/>
@@ -1191,7 +1197,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="n">
         <v>56</v>
       </c>
@@ -1201,7 +1207,7 @@
       <c r="C2" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>53</v>
       </c>
       <c r="E2" s="8" t="n">
@@ -1228,23 +1234,23 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" s="12" customFormat="true" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="n">
+    <row r="4" s="13" customFormat="true" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="C4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="10" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1255,7 +1261,7 @@
       <c r="B5" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="11" t="s">
         <v>17</v>
       </c>
       <c r="D5" s="8" t="s">
@@ -1264,15 +1270,37 @@
       <c r="E5" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="8" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="n">
+        <v>731</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" display="https://leetcode.com/problems/interval-list-intersections/"/>
-    <hyperlink ref="D4" r:id="rId2" display="https://leetcode.com/problems/insert-interval/"/>
-    <hyperlink ref="D5" r:id="rId3" display="https://leetcode.com/problems/remove-covered-intervals/"/>
+    <hyperlink ref="D2" r:id="rId1" display="https://leetcode.com/problems/merge-intervals/"/>
+    <hyperlink ref="D3" r:id="rId2" display="https://leetcode.com/problems/interval-list-intersections/"/>
+    <hyperlink ref="D4" r:id="rId3" display="https://leetcode.com/problems/insert-interval/"/>
+    <hyperlink ref="D5" r:id="rId4" display="https://leetcode.com/problems/remove-covered-intervals/"/>
+    <hyperlink ref="D6" r:id="rId5" display="https://leetcode.com/problems/my-calendar-ii/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Done with day 28
</commit_message>
<xml_diff>
--- a/3.Problems for Revision.xlsx
+++ b/3.Problems for Revision.xlsx
@@ -223,7 +223,7 @@
     <t xml:space="preserve">25 &amp; 26</t>
   </si>
   <si>
-    <t xml:space="preserve">Line Sweep Algo explained</t>
+    <t xml:space="preserve">Line Sweep Algo</t>
   </si>
 </sst>
 </file>
@@ -397,7 +397,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -431,10 +431,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1207,7 +1203,7 @@
       <c r="C2" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>53</v>
       </c>
       <c r="E2" s="8" t="n">
@@ -1234,23 +1230,23 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" s="13" customFormat="true" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+    <row r="4" s="12" customFormat="true" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="n">
         <v>57</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="12" t="s">
+      <c r="C4" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1261,7 +1257,7 @@
       <c r="B5" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>17</v>
       </c>
       <c r="D5" s="8" t="s">
@@ -1281,7 +1277,7 @@
       <c r="B6" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>17</v>
       </c>
       <c r="D6" s="8" t="s">

</xml_diff>

<commit_message>
Done with day 30 - Interval Pattern
</commit_message>
<xml_diff>
--- a/3.Problems for Revision.xlsx
+++ b/3.Problems for Revision.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -236,6 +236,15 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/my-calendar-iii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Stream as Disjoint Intervals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/data-stream-as-disjoint-intervals/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tree Set</t>
   </si>
 </sst>
 </file>
@@ -409,7 +418,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -460,6 +469,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -757,7 +770,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>1365</v>
       </c>
@@ -842,7 +855,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>1886</v>
       </c>
@@ -1173,13 +1186,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="18.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="32.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="35.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="8" width="18.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="63.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="68.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="8" width="18.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="8" width="59.26"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="8" width="11.53"/>
@@ -1340,6 +1353,26 @@
       </c>
       <c r="F8" s="8" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="n">
+        <v>352</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1351,6 +1384,7 @@
     <hyperlink ref="D6" r:id="rId5" display="https://leetcode.com/problems/my-calendar-ii/"/>
     <hyperlink ref="D7" r:id="rId6" display="https://leetcode.com/problems/my-calendar-i/"/>
     <hyperlink ref="D8" r:id="rId7" display="https://leetcode.com/problems/my-calendar-iii/"/>
+    <hyperlink ref="D9" r:id="rId8" display="https://leetcode.com/problems/data-stream-as-disjoint-intervals/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Start with In-Place LinkedList manipulation Pattern
</commit_message>
<xml_diff>
--- a/3.Problems for Revision.xlsx
+++ b/3.Problems for Revision.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Two Pointers" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Fast&amp;Slow Pointers" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Sliding Window" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Intervals" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Linked List - In-Place Manipula" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="74">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -418,7 +419,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -471,8 +472,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -770,7 +775,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>1365</v>
       </c>
@@ -855,7 +860,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>1886</v>
       </c>
@@ -1359,7 +1364,7 @@
       <c r="A9" s="8" t="n">
         <v>352</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="8" t="s">
         <v>71</v>
       </c>
       <c r="C9" s="8" t="s">
@@ -1394,4 +1399,55 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="16.15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="13" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="13" width="39.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="13" width="15.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="13" width="53.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="5" style="13" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="13" width="55.11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="13" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="20.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D7" s="14"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add NOTE to help solve the problems
</commit_message>
<xml_diff>
--- a/3.Problems for Revision.xlsx
+++ b/3.Problems for Revision.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="86">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -279,6 +279,27 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/reorder-list/</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Comic Sans MS"/>
+        <family val="4"/>
+      </rPr>
+      <t xml:space="preserve">NOTE:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Comic Sans MS"/>
+        <family val="4"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Check whether the problem requires a dummy node or not, check code for even and odd length Linked Lists, check what happens of head == null (empty list) and head.next == null (single node).</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -288,7 +309,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -398,6 +419,12 @@
       <family val="4"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -540,11 +567,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -555,16 +582,16 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1493,7 +1520,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="16.15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="13" width="11.53"/>
@@ -1538,13 +1565,13 @@
       <c r="D2" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="17" t="n">
+      <c r="E2" s="15" t="n">
         <v>32</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="G2" s="18"/>
+      <c r="G2" s="17"/>
     </row>
     <row r="3" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="n">
@@ -1559,13 +1586,13 @@
       <c r="D3" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="E3" s="15" t="n">
         <v>32</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="18"/>
     </row>
     <row r="4" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="n">
@@ -1580,15 +1607,15 @@
       <c r="D4" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="E4" s="17" t="n">
+      <c r="E4" s="15" t="n">
         <v>33</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="19"/>
-    </row>
-    <row r="5" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G4" s="18"/>
+    </row>
+    <row r="5" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="n">
         <v>143</v>
       </c>
@@ -1601,13 +1628,18 @@
       <c r="D5" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="15" t="n">
         <v>33</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="G5" s="0"/>
+      <c r="G5" s="18"/>
+    </row>
+    <row r="20" customFormat="false" ht="81.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D20" s="19" t="s">
+        <v>85</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Solve N-Queens - Leetcode Hard
</commit_message>
<xml_diff>
--- a/3.Problems for Revision.xlsx
+++ b/3.Problems for Revision.xlsx
@@ -5,14 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
-    <sheet name="Two Pointers" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Fast&amp;Slow Pointers" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Sliding Window" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Intervals" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Linked List - In-Place Manipula" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Practice Problems (Kunal + Anuj" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Two Pointers" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Fast&amp;Slow Pointers" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Sliding Window" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Intervals" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Linked List - In-Place Manipula" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="125">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -38,15 +39,78 @@
     <t xml:space="preserve">LeetCode URL</t>
   </si>
   <si>
+    <t xml:space="preserve">Video URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pascal’s Triangle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Easy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/pascals-triangle/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youtu.be/ELo7RR-Isjk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pascal’s Triangle II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/pascals-triangle-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3Sum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/3sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youtu.be/rM9EthMlXnw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3Sum Closest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/3sum-closest/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letter Combinations of a Phone Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/letter-combinations-of-a-phone-number/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youtu.be/9ByWqPzfXDU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resursion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Queens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/n-queens/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youtu.be/nC1rbW2YSz0</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resource</t>
   </si>
   <si>
     <t xml:space="preserve">Split Array Largest Sum</t>
   </si>
   <si>
-    <t xml:space="preserve">Hard</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://leetcode.com/problems/split-array-largest-sum/description/</t>
   </si>
   <si>
@@ -56,9 +120,6 @@
     <t xml:space="preserve">How Many Numbers Are Smaller Than the Current Number</t>
   </si>
   <si>
-    <t xml:space="preserve">Easy</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://leetcode.com/problems/how-many-numbers-are-smaller-than-the-current-number/description/</t>
   </si>
   <si>
@@ -75,9 +136,6 @@
   </si>
   <si>
     <t xml:space="preserve">Lowest Common Ancestor of a Binary Tree III</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medium</t>
   </si>
   <si>
     <t xml:space="preserve">https://neetcode.io/problems/lowest-common-ancestor-of-a-binary-tree-iii</t>
@@ -484,6 +542,21 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="medium">
         <color rgb="FFCCCCCC"/>
       </left>
@@ -495,21 +568,6 @@
       </top>
       <bottom style="medium">
         <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -542,20 +600,32 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -571,11 +641,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -603,15 +673,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -623,19 +693,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -889,151 +959,314 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15.85" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="67.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="70.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.54"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="20.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>118</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>119</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="https://leetcode.com/problems/pascals-triangle/"/>
+    <hyperlink ref="E2" r:id="rId2" display="https://youtu.be/ELo7RR-Isjk"/>
+    <hyperlink ref="D3" r:id="rId3" display="https://leetcode.com/problems/pascals-triangle-ii/"/>
+    <hyperlink ref="D4" r:id="rId4" display="https://leetcode.com/problems/3sum/"/>
+    <hyperlink ref="E4" r:id="rId5" display="https://youtu.be/rM9EthMlXnw"/>
+    <hyperlink ref="D5" r:id="rId6" display="https://leetcode.com/problems/3sum-closest/"/>
+    <hyperlink ref="E5" r:id="rId7" display="https://youtu.be/rM9EthMlXnw"/>
+    <hyperlink ref="D6" r:id="rId8" display="https://leetcode.com/problems/letter-combinations-of-a-phone-number/"/>
+    <hyperlink ref="E6" r:id="rId9" display="https://youtu.be/9ByWqPzfXDU"/>
+    <hyperlink ref="D7" r:id="rId10" display="https://leetcode.com/problems/n-queens/"/>
+    <hyperlink ref="E7" r:id="rId11" display="https://youtu.be/nC1rbW2YSz0"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="129.5625" defaultRowHeight="19.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="69.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="85.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="129.33"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="129.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="6.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="69.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="9.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="85.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="129.33"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="4" width="129.56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
+      <c r="E1" s="5" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="4" t="n">
         <v>410</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="B2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="n">
+        <v>1365</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
-        <v>1365</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>12</v>
+      <c r="D3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="4" t="n">
         <v>246</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>15</v>
+      <c r="B4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="4" t="n">
         <v>1650</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>15</v>
+      <c r="B5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="4" t="n">
         <v>151</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>21</v>
+      <c r="B6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="4" t="n">
         <v>557</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>12</v>
+      <c r="B7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="4" t="n">
         <v>1886</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>12</v>
+      <c r="B8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1060,7 +1293,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1068,96 +1301,96 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="129.5625" defaultRowHeight="19.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="69.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="87.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.44"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="129.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="6.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="69.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="9.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="87.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="11.44"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="4" width="129.56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>26</v>
+      <c r="E1" s="5" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="8" t="n">
         <v>142</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="1" t="n">
+      <c r="B2" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="8" t="n">
         <v>287</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="1" t="n">
+      <c r="B3" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="4" t="n">
         <v>234</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" s="1" t="n">
+      <c r="B4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="4" t="n">
         <v>457</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="1" t="n">
+      <c r="B5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -1172,7 +1405,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1180,208 +1413,208 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="19.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="63.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="67.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="43.9"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="8.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="63.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="67.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="13.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="4" width="43.9"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="4" width="8.88"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="20.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="39.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+      <c r="E1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="n">
         <v>209</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="B2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="n">
+        <v>2461</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>187</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="n">
+        <v>904</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="39.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>1838</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="39.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
-        <v>2461</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="39.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="20.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
-        <v>187</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="20.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
-        <v>904</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="39.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="n">
-        <v>1838</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="39.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
+      <c r="F7" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="n">
         <v>424</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" s="1" t="n">
+      <c r="B8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>51</v>
+      <c r="F8" s="9" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="4" t="n">
         <v>1493</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>55</v>
+      <c r="B9" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="4" t="n">
         <v>1004</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>51</v>
+      <c r="B10" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0"/>
-      <c r="B11" s="0"/>
-      <c r="C11" s="0"/>
-      <c r="D11" s="0"/>
-      <c r="E11" s="0"/>
-      <c r="F11" s="0"/>
-      <c r="G11" s="8"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1398,7 +1631,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1406,190 +1639,190 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="9" width="18.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="9" width="35.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="9" width="18.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="9" width="68.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="9" width="18.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="9" width="59.26"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="9" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="18.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="35.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="12" width="18.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="68.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="12" width="18.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="12" width="59.26"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="12" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
+      <c r="E1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="n">
+      <c r="A2" s="12" t="n">
         <v>56</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="9" t="n">
+      <c r="B2" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="F2" s="9" t="s">
-        <v>61</v>
+      <c r="F2" s="12" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="n">
+      <c r="A3" s="12" t="n">
         <v>986</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E3" s="9" t="n">
+      <c r="B3" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" s="12" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="4" s="13" customFormat="true" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+    <row r="4" s="16" customFormat="true" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="n">
         <v>57</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="E4" s="11" t="n">
+      <c r="B4" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>66</v>
+      <c r="F4" s="13" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="12" t="n">
         <v>1288</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="9" t="n">
+      <c r="B5" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>69</v>
+      <c r="F5" s="12" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="12" t="n">
         <v>731</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>73</v>
+      <c r="B6" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="12" t="n">
         <v>729</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" s="9" t="n">
+      <c r="B7" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="E7" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="F7" s="9" t="s">
-        <v>73</v>
+      <c r="F7" s="12" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="12" t="n">
         <v>732</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="9" t="n">
+      <c r="B8" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>73</v>
+      <c r="F8" s="12" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="12" t="n">
         <v>352</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E9" s="9" t="n">
+      <c r="B9" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>80</v>
+      <c r="F9" s="12" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1613,7 +1846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1621,203 +1854,203 @@
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="16.15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="14" width="8.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="14" width="37.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="14" width="23.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="14" width="72.65"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="5" style="14" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="14" width="48.38"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="14" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="8.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="37.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="17" width="23.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="17" width="72.65"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="5" style="17" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="17" width="48.38"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="17" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="20.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="E1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="18" t="n">
+        <v>206</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="E2" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="G2" s="21"/>
+    </row>
+    <row r="3" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="n">
+        <v>203</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="G3" s="21"/>
+    </row>
+    <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="n">
+        <v>92</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>33</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="G4" s="21"/>
+    </row>
+    <row r="5" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="n">
+        <v>143</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>33</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="G5" s="21"/>
+    </row>
+    <row r="6" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="n">
+        <v>328</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>34</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G6" s="22"/>
+    </row>
+    <row r="7" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="n">
+        <v>725</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="E7" s="19" t="n">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="33.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="15" t="n">
-        <v>206</v>
-      </c>
-      <c r="B2" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="C2" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="G2" s="18"/>
-    </row>
-    <row r="3" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="n">
-        <v>203</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="E3" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G3" s="18"/>
-    </row>
-    <row r="4" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="n">
-        <v>92</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" s="16" t="n">
-        <v>33</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="G4" s="18"/>
-    </row>
-    <row r="5" customFormat="false" ht="33.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="n">
-        <v>143</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <v>33</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="G5" s="18"/>
-    </row>
-    <row r="6" customFormat="false" ht="33.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="n">
-        <v>328</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>34</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="G6" s="19"/>
-    </row>
-    <row r="7" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="n">
-        <v>725</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>35</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="G7" s="19"/>
-    </row>
-    <row r="8" customFormat="false" ht="20.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="n">
+      <c r="F7" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="G7" s="22"/>
+    </row>
+    <row r="8" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="n">
         <v>25</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="E8" s="20" t="n">
+      <c r="B8" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" s="23" t="n">
         <v>36</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="23"/>
-    </row>
-    <row r="9" customFormat="false" ht="39.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
+      <c r="F8" s="25"/>
+      <c r="G8" s="26"/>
+    </row>
+    <row r="9" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="n">
         <v>2074</v>
       </c>
-      <c r="B9" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>103</v>
-      </c>
-      <c r="E9" s="20" t="n">
+      <c r="B9" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="E9" s="23" t="n">
         <v>37</v>
       </c>
-      <c r="F9" s="22" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="48.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D20" s="14" t="s">
-        <v>105</v>
+      <c r="F9" s="25" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D20" s="17" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add N-Queens and Sudoku solver in Excel
</commit_message>
<xml_diff>
--- a/3.Problems for Revision.xlsx
+++ b/3.Problems for Revision.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="128">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t xml:space="preserve">Resursion + Backtracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sudoku Solver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/sudoku-solver/</t>
   </si>
   <si>
     <t xml:space="preserve">Resource</t>
@@ -962,7 +968,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15.85" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.78"/>
@@ -1099,6 +1105,26 @@
         <v>26</v>
       </c>
     </row>
+    <row r="8" customFormat="false" ht="20.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="https://leetcode.com/problems/pascals-triangle/"/>
@@ -1112,6 +1138,8 @@
     <hyperlink ref="E6" r:id="rId9" display="https://youtu.be/9ByWqPzfXDU"/>
     <hyperlink ref="D7" r:id="rId10" display="https://leetcode.com/problems/n-queens/"/>
     <hyperlink ref="E7" r:id="rId11" display="https://youtu.be/nC1rbW2YSz0"/>
+    <hyperlink ref="D8" r:id="rId12" display="https://leetcode.com/problems/sudoku-solver/"/>
+    <hyperlink ref="E8" r:id="rId13" display="https://youtu.be/nC1rbW2YSz0"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1153,7 +1181,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1161,16 +1189,16 @@
         <v>410</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>23</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1178,16 +1206,16 @@
         <v>1365</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1195,16 +1223,16 @@
         <v>246</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1212,16 +1240,16 @@
         <v>1650</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1229,16 +1257,16 @@
         <v>151</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1246,16 +1274,16 @@
         <v>557</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1263,16 +1291,16 @@
         <v>1886</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1329,7 +1357,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1337,13 +1365,13 @@
         <v>142</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>8</v>
@@ -1354,13 +1382,13 @@
         <v>287</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>9</v>
@@ -1371,13 +1399,13 @@
         <v>234</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>9</v>
@@ -1388,13 +1416,13 @@
         <v>457</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>11</v>
@@ -1442,10 +1470,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1453,13 +1481,13 @@
         <v>209</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>13</v>
@@ -1470,13 +1498,13 @@
         <v>2461</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>13</v>
@@ -1487,13 +1515,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>14</v>
@@ -1504,13 +1532,13 @@
         <v>187</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>15</v>
@@ -1521,13 +1549,13 @@
         <v>904</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>16</v>
@@ -1538,19 +1566,19 @@
         <v>1838</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>17</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1558,19 +1586,19 @@
         <v>424</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>18</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1578,19 +1606,19 @@
         <v>1493</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1598,19 +1626,19 @@
         <v>1004</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>74</v>
-      </c>
       <c r="F10" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1668,10 +1696,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1679,19 +1707,19 @@
         <v>56</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E2" s="12" t="n">
         <v>21</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1699,13 +1727,13 @@
         <v>986</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E3" s="12" t="n">
         <v>22</v>
@@ -1716,19 +1744,19 @@
         <v>57</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>23</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1736,19 +1764,19 @@
         <v>1288</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>24</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1756,19 +1784,19 @@
         <v>731</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1776,19 +1804,19 @@
         <v>729</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E7" s="12" t="n">
         <v>27</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1796,19 +1824,19 @@
         <v>732</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>29</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1816,19 +1844,19 @@
         <v>352</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E9" s="12" t="n">
         <v>30</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1883,10 +1911,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1894,19 +1922,19 @@
         <v>206</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E2" s="19" t="n">
         <v>32</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G2" s="21"/>
     </row>
@@ -1915,19 +1943,19 @@
         <v>203</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C3" s="19" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E3" s="19" t="n">
         <v>32</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G3" s="21"/>
     </row>
@@ -1936,19 +1964,19 @@
         <v>92</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E4" s="19" t="n">
         <v>33</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G4" s="21"/>
     </row>
@@ -1957,19 +1985,19 @@
         <v>143</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C5" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E5" s="19" t="n">
         <v>33</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G5" s="21"/>
     </row>
@@ -1978,19 +2006,19 @@
         <v>328</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E6" s="19" t="n">
         <v>34</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G6" s="22"/>
     </row>
@@ -1999,19 +2027,19 @@
         <v>725</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E7" s="19" t="n">
         <v>35</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G7" s="22"/>
     </row>
@@ -2020,13 +2048,13 @@
         <v>25</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C8" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E8" s="23" t="n">
         <v>36</v>
@@ -2039,24 +2067,24 @@
         <v>2074</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E9" s="23" t="n">
         <v>37</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D20" s="17" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve Leetcode 36 Valid Sudoku
</commit_message>
<xml_diff>
--- a/3.Problems for Revision.xlsx
+++ b/3.Problems for Revision.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="131">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -112,6 +112,15 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/sudoku-solver/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid Sudoku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/valid-sudoku/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Similar to Leetcode 37</t>
   </si>
   <si>
     <t xml:space="preserve">Resource</t>
@@ -968,7 +977,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15.85" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.78"/>
@@ -1105,7 +1114,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="20.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>37</v>
       </c>
@@ -1123,6 +1132,23 @@
       </c>
       <c r="F8" s="1" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1140,6 +1166,7 @@
     <hyperlink ref="E7" r:id="rId11" display="https://youtu.be/nC1rbW2YSz0"/>
     <hyperlink ref="D8" r:id="rId12" display="https://leetcode.com/problems/sudoku-solver/"/>
     <hyperlink ref="E8" r:id="rId13" display="https://youtu.be/nC1rbW2YSz0"/>
+    <hyperlink ref="D9" r:id="rId14" display="https://leetcode.com/problems/valid-sudoku/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1181,7 +1208,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1189,16 +1216,16 @@
         <v>410</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>23</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1206,16 +1233,16 @@
         <v>1365</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1223,16 +1250,16 @@
         <v>246</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1240,16 +1267,16 @@
         <v>1650</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1257,16 +1284,16 @@
         <v>151</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1274,16 +1301,16 @@
         <v>557</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1291,16 +1318,16 @@
         <v>1886</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1357,7 +1384,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1365,13 +1392,13 @@
         <v>142</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>8</v>
@@ -1382,13 +1409,13 @@
         <v>287</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>9</v>
@@ -1399,13 +1426,13 @@
         <v>234</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>9</v>
@@ -1416,13 +1443,13 @@
         <v>457</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>11</v>
@@ -1470,10 +1497,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1481,13 +1508,13 @@
         <v>209</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>13</v>
@@ -1498,13 +1525,13 @@
         <v>2461</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>13</v>
@@ -1515,13 +1542,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>14</v>
@@ -1532,13 +1559,13 @@
         <v>187</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>15</v>
@@ -1549,13 +1576,13 @@
         <v>904</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>16</v>
@@ -1566,19 +1593,19 @@
         <v>1838</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>17</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1586,19 +1613,19 @@
         <v>424</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>18</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1606,19 +1633,19 @@
         <v>1493</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1626,19 +1653,19 @@
         <v>1004</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="F10" s="10" t="s">
         <v>76</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1696,10 +1723,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1707,19 +1734,19 @@
         <v>56</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E2" s="12" t="n">
         <v>21</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1727,13 +1754,13 @@
         <v>986</v>
       </c>
       <c r="B3" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>81</v>
-      </c>
       <c r="D3" s="12" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E3" s="12" t="n">
         <v>22</v>
@@ -1744,19 +1771,19 @@
         <v>57</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>23</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1764,19 +1791,19 @@
         <v>1288</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>24</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1784,19 +1811,19 @@
         <v>731</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1804,19 +1831,19 @@
         <v>729</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E7" s="12" t="n">
         <v>27</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1824,19 +1851,19 @@
         <v>732</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>29</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1844,19 +1871,19 @@
         <v>352</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E9" s="12" t="n">
         <v>30</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1911,10 +1938,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1922,19 +1949,19 @@
         <v>206</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E2" s="19" t="n">
         <v>32</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G2" s="21"/>
     </row>
@@ -1943,19 +1970,19 @@
         <v>203</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C3" s="19" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E3" s="19" t="n">
         <v>32</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G3" s="21"/>
     </row>
@@ -1964,19 +1991,19 @@
         <v>92</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E4" s="19" t="n">
         <v>33</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G4" s="21"/>
     </row>
@@ -1985,19 +2012,19 @@
         <v>143</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C5" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E5" s="19" t="n">
         <v>33</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G5" s="21"/>
     </row>
@@ -2006,19 +2033,19 @@
         <v>328</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E6" s="19" t="n">
         <v>34</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="G6" s="22"/>
     </row>
@@ -2027,19 +2054,19 @@
         <v>725</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E7" s="19" t="n">
         <v>35</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G7" s="22"/>
     </row>
@@ -2048,13 +2075,13 @@
         <v>25</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C8" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E8" s="23" t="n">
         <v>36</v>
@@ -2067,24 +2094,24 @@
         <v>2074</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E9" s="23" t="n">
         <v>37</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D20" s="17" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>